<commit_message>
Deploying to gh-pages from @ Narendra920/pdd@53ffdb49fa1b0bc9f26ffcb2c0145d089d9279d3 🚀
</commit_message>
<xml_diff>
--- a/android-reports/latest/appium-report.xlsx
+++ b/android-reports/latest/appium-report.xlsx
@@ -545,7 +545,7 @@
         <v>6</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -594,7 +594,7 @@
         <v>17</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ Narendra920/pdd@5250cafdf41ceb07dcd3c96492cbb9628284642d 🚀
</commit_message>
<xml_diff>
--- a/android-reports/latest/appium-report.xlsx
+++ b/android-reports/latest/appium-report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>Metric</t>
   </si>
@@ -33,7 +33,7 @@
     <t>Pass Rate</t>
   </si>
   <si>
-    <t>0.00%</t>
+    <t>0%</t>
   </si>
   <si>
     <t>Category</t>
@@ -51,9 +51,6 @@
     <t>Duration (ms)</t>
   </si>
   <si>
-    <t>Fatal</t>
-  </si>
-  <si>
     <t>Title</t>
   </si>
   <si>
@@ -61,15 +58,6 @@
   </si>
   <si>
     <t>Error</t>
-  </si>
-  <si>
-    <t>[Fatal-T1] Setup/Appium Crash</t>
-  </si>
-  <si>
-    <t>failed</t>
-  </si>
-  <si>
-    <t>WebDriver session failed to initialize or crashed.</t>
   </si>
 </sst>
 </file>
@@ -465,7 +453,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -481,7 +469,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -500,7 +488,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -528,26 +516,6 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -556,7 +524,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -571,33 +539,16 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>13</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
       </c>
       <c r="D1" t="s">
         <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2">
         <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>